<commit_message>
adding map and some minor corrections
</commit_message>
<xml_diff>
--- a/data/Finland_resampling2025_Sites.xlsx
+++ b/data/Finland_resampling2025_Sites.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\Documents\GitHub\finland_ew_time_analysis\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59AC5AC9-D23A-4738-B838-318D9884D828}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC93C6B2-E6B2-4D38-967A-68F6C10EF77A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{62381CB3-6983-4B4B-80E0-EF394FFF3EEF}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1627" uniqueCount="213">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2317" uniqueCount="283">
   <si>
     <t>site_name</t>
   </si>
@@ -678,6 +678,216 @@
   </si>
   <si>
     <t>kilpisjarvi_93_9</t>
+  </si>
+  <si>
+    <t>Tvarminne_8</t>
+  </si>
+  <si>
+    <t>Tvarminne_8_1</t>
+  </si>
+  <si>
+    <t>Tvarminne_8_2</t>
+  </si>
+  <si>
+    <t>Tvarminne_8_3</t>
+  </si>
+  <si>
+    <t>Tvarminne_8_4</t>
+  </si>
+  <si>
+    <t>Tvarminne_8_5</t>
+  </si>
+  <si>
+    <t>Tvarminne_8_6</t>
+  </si>
+  <si>
+    <t>Tvarminne_8_7</t>
+  </si>
+  <si>
+    <t>Tvarminne_8_8</t>
+  </si>
+  <si>
+    <t>Tvarminne_8_9</t>
+  </si>
+  <si>
+    <t>recent clear cut, baby birch and spruce (about 2 yo). Small streams close to the site.</t>
+  </si>
+  <si>
+    <t>It rained during sampling</t>
+  </si>
+  <si>
+    <t>Sylvain GERARD, Alberto PIRIS</t>
+  </si>
+  <si>
+    <t>Tvarminne_627</t>
+  </si>
+  <si>
+    <t>Tvarminne_627_1</t>
+  </si>
+  <si>
+    <t>Tvarminne_627_2</t>
+  </si>
+  <si>
+    <t>Tvarminne_627_3</t>
+  </si>
+  <si>
+    <t>Tvarminne_627_4</t>
+  </si>
+  <si>
+    <t>Tvarminne_627_5</t>
+  </si>
+  <si>
+    <t>Tvarminne_627_6</t>
+  </si>
+  <si>
+    <t>Tvarminne_627_7</t>
+  </si>
+  <si>
+    <t>Tvarminne_627_8</t>
+  </si>
+  <si>
+    <t>Tvarminne_627_9</t>
+  </si>
+  <si>
+    <t>birch forest, not really dense. Some pine and spruce here and there. No understory.</t>
+  </si>
+  <si>
+    <t>plot 1 not geolocalised in Erin data</t>
+  </si>
+  <si>
+    <t>Tvarminne_34</t>
+  </si>
+  <si>
+    <t>Tvarminne_34_1</t>
+  </si>
+  <si>
+    <t>Tvarminne_34_2</t>
+  </si>
+  <si>
+    <t>Tvarminne_34_3</t>
+  </si>
+  <si>
+    <t>Tvarminne_34_4</t>
+  </si>
+  <si>
+    <t>Tvarminne_34_5</t>
+  </si>
+  <si>
+    <t>Tvarminne_34_6</t>
+  </si>
+  <si>
+    <t>Tvarminne_34_7</t>
+  </si>
+  <si>
+    <t>Tvarminne_34_8</t>
+  </si>
+  <si>
+    <t>Tvarminne_34_9</t>
+  </si>
+  <si>
+    <t>spruce forest, no understory</t>
+  </si>
+  <si>
+    <t>not too far from clear cut</t>
+  </si>
+  <si>
+    <t>Tvarminne_61</t>
+  </si>
+  <si>
+    <t>Tvarminne_61_1</t>
+  </si>
+  <si>
+    <t>Tvarminne_61_2</t>
+  </si>
+  <si>
+    <t>Tvarminne_61_3</t>
+  </si>
+  <si>
+    <t>Tvarminne_61_4</t>
+  </si>
+  <si>
+    <t>Tvarminne_61_5</t>
+  </si>
+  <si>
+    <t>Tvarminne_61_6</t>
+  </si>
+  <si>
+    <t>Tvarminne_61_7</t>
+  </si>
+  <si>
+    <t>Tvarminne_61_8</t>
+  </si>
+  <si>
+    <t>Tvarminne_61_9</t>
+  </si>
+  <si>
+    <t>mixed forest, birch and spruce. No understory</t>
+  </si>
+  <si>
+    <t>we sampled in a birch patch but the forest was globally more dominated by spruce. Close to clear cut</t>
+  </si>
+  <si>
+    <t>Tvarminne_11</t>
+  </si>
+  <si>
+    <t>Tvarminne_11_1</t>
+  </si>
+  <si>
+    <t>Tvarminne_11_2</t>
+  </si>
+  <si>
+    <t>Tvarminne_11_3</t>
+  </si>
+  <si>
+    <t>Tvarminne_11_4</t>
+  </si>
+  <si>
+    <t>Tvarminne_11_5</t>
+  </si>
+  <si>
+    <t>Tvarminne_11_6</t>
+  </si>
+  <si>
+    <t>Tvarminne_11_7</t>
+  </si>
+  <si>
+    <t>Tvarminne_11_8</t>
+  </si>
+  <si>
+    <t>Tvarminne_11_9</t>
+  </si>
+  <si>
+    <t>Tvarminne_60</t>
+  </si>
+  <si>
+    <t>Tvarminne_60_1</t>
+  </si>
+  <si>
+    <t>Tvarminne_60_2</t>
+  </si>
+  <si>
+    <t>Tvarminne_60_3</t>
+  </si>
+  <si>
+    <t>Tvarminne_60_4</t>
+  </si>
+  <si>
+    <t>Tvarminne_60_5</t>
+  </si>
+  <si>
+    <t>Tvarminne_60_6</t>
+  </si>
+  <si>
+    <t>Tvarminne_60_7</t>
+  </si>
+  <si>
+    <t>Tvarminne_60_8</t>
+  </si>
+  <si>
+    <t>Tvarminne_60_9</t>
+  </si>
+  <si>
+    <t>mixed forest, quite dense, birch and spruce</t>
   </si>
 </sst>
 </file>
@@ -1063,7 +1273,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1DCF7B1D-30EB-41FA-B0BA-2D9928994D79}">
-  <dimension ref="A1:K227"/>
+  <dimension ref="A1:K317"/>
   <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.6640625" customWidth="1"/>
@@ -7860,6 +8070,2670 @@
         <v>125</v>
       </c>
     </row>
+    <row r="228" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A228" t="s">
+        <v>213</v>
+      </c>
+      <c r="B228" t="s">
+        <v>214</v>
+      </c>
+      <c r="C228" t="s">
+        <v>3</v>
+      </c>
+      <c r="D228" t="s">
+        <v>70</v>
+      </c>
+      <c r="E228">
+        <v>20260504</v>
+      </c>
+      <c r="F228">
+        <v>59.981280900000002</v>
+      </c>
+      <c r="G228">
+        <v>23.3642228</v>
+      </c>
+      <c r="H228" t="s">
+        <v>223</v>
+      </c>
+      <c r="I228" t="s">
+        <v>224</v>
+      </c>
+      <c r="J228" t="s">
+        <v>225</v>
+      </c>
+      <c r="K228" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="229" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A229" t="s">
+        <v>213</v>
+      </c>
+      <c r="B229" t="s">
+        <v>214</v>
+      </c>
+      <c r="C229" t="s">
+        <v>6</v>
+      </c>
+      <c r="D229" t="s">
+        <v>123</v>
+      </c>
+      <c r="E229">
+        <v>20260504</v>
+      </c>
+      <c r="F229">
+        <v>59.981280900000002</v>
+      </c>
+      <c r="G229">
+        <v>23.3642228</v>
+      </c>
+      <c r="H229" t="s">
+        <v>223</v>
+      </c>
+      <c r="I229" t="s">
+        <v>224</v>
+      </c>
+      <c r="J229" t="s">
+        <v>225</v>
+      </c>
+      <c r="K229" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="230" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A230" t="s">
+        <v>213</v>
+      </c>
+      <c r="B230" t="s">
+        <v>215</v>
+      </c>
+      <c r="C230" t="s">
+        <v>3</v>
+      </c>
+      <c r="D230" t="s">
+        <v>70</v>
+      </c>
+      <c r="E230">
+        <v>20260504</v>
+      </c>
+      <c r="H230" t="s">
+        <v>223</v>
+      </c>
+      <c r="I230" t="s">
+        <v>224</v>
+      </c>
+      <c r="J230" t="s">
+        <v>225</v>
+      </c>
+      <c r="K230" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="231" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A231" t="s">
+        <v>213</v>
+      </c>
+      <c r="B231" t="s">
+        <v>215</v>
+      </c>
+      <c r="C231" t="s">
+        <v>6</v>
+      </c>
+      <c r="D231" t="s">
+        <v>123</v>
+      </c>
+      <c r="E231">
+        <v>20260504</v>
+      </c>
+      <c r="H231" t="s">
+        <v>223</v>
+      </c>
+      <c r="I231" t="s">
+        <v>224</v>
+      </c>
+      <c r="J231" t="s">
+        <v>225</v>
+      </c>
+      <c r="K231" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="232" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A232" t="s">
+        <v>213</v>
+      </c>
+      <c r="B232" t="s">
+        <v>216</v>
+      </c>
+      <c r="C232" t="s">
+        <v>3</v>
+      </c>
+      <c r="D232" t="s">
+        <v>70</v>
+      </c>
+      <c r="E232">
+        <v>20260504</v>
+      </c>
+      <c r="H232" t="s">
+        <v>223</v>
+      </c>
+      <c r="I232" t="s">
+        <v>224</v>
+      </c>
+      <c r="J232" t="s">
+        <v>225</v>
+      </c>
+      <c r="K232" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="233" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A233" t="s">
+        <v>213</v>
+      </c>
+      <c r="B233" t="s">
+        <v>216</v>
+      </c>
+      <c r="C233" t="s">
+        <v>6</v>
+      </c>
+      <c r="D233" t="s">
+        <v>123</v>
+      </c>
+      <c r="E233">
+        <v>20260504</v>
+      </c>
+      <c r="H233" t="s">
+        <v>223</v>
+      </c>
+      <c r="I233" t="s">
+        <v>224</v>
+      </c>
+      <c r="J233" t="s">
+        <v>225</v>
+      </c>
+      <c r="K233" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="234" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A234" t="s">
+        <v>213</v>
+      </c>
+      <c r="B234" t="s">
+        <v>217</v>
+      </c>
+      <c r="C234" t="s">
+        <v>3</v>
+      </c>
+      <c r="D234" t="s">
+        <v>70</v>
+      </c>
+      <c r="E234">
+        <v>20260504</v>
+      </c>
+      <c r="H234" t="s">
+        <v>223</v>
+      </c>
+      <c r="I234" t="s">
+        <v>224</v>
+      </c>
+      <c r="J234" t="s">
+        <v>225</v>
+      </c>
+      <c r="K234" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="235" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A235" t="s">
+        <v>213</v>
+      </c>
+      <c r="B235" t="s">
+        <v>217</v>
+      </c>
+      <c r="C235" t="s">
+        <v>6</v>
+      </c>
+      <c r="D235" t="s">
+        <v>123</v>
+      </c>
+      <c r="E235">
+        <v>20260504</v>
+      </c>
+      <c r="H235" t="s">
+        <v>223</v>
+      </c>
+      <c r="I235" t="s">
+        <v>224</v>
+      </c>
+      <c r="J235" t="s">
+        <v>225</v>
+      </c>
+      <c r="K235" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="236" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A236" t="s">
+        <v>213</v>
+      </c>
+      <c r="B236" t="s">
+        <v>218</v>
+      </c>
+      <c r="C236" t="s">
+        <v>3</v>
+      </c>
+      <c r="D236" t="s">
+        <v>70</v>
+      </c>
+      <c r="E236">
+        <v>20260504</v>
+      </c>
+      <c r="H236" t="s">
+        <v>223</v>
+      </c>
+      <c r="I236" t="s">
+        <v>224</v>
+      </c>
+      <c r="J236" t="s">
+        <v>225</v>
+      </c>
+      <c r="K236" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="237" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A237" t="s">
+        <v>213</v>
+      </c>
+      <c r="B237" t="s">
+        <v>218</v>
+      </c>
+      <c r="C237" t="s">
+        <v>6</v>
+      </c>
+      <c r="D237" t="s">
+        <v>123</v>
+      </c>
+      <c r="E237">
+        <v>20260504</v>
+      </c>
+      <c r="H237" t="s">
+        <v>223</v>
+      </c>
+      <c r="I237" t="s">
+        <v>224</v>
+      </c>
+      <c r="J237" t="s">
+        <v>225</v>
+      </c>
+      <c r="K237" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="238" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A238" t="s">
+        <v>213</v>
+      </c>
+      <c r="B238" t="s">
+        <v>219</v>
+      </c>
+      <c r="C238" t="s">
+        <v>3</v>
+      </c>
+      <c r="D238" t="s">
+        <v>70</v>
+      </c>
+      <c r="E238">
+        <v>20260504</v>
+      </c>
+      <c r="F238">
+        <v>59.981255300000001</v>
+      </c>
+      <c r="G238">
+        <v>23.3646329</v>
+      </c>
+      <c r="H238" t="s">
+        <v>223</v>
+      </c>
+      <c r="I238" t="s">
+        <v>224</v>
+      </c>
+      <c r="J238" t="s">
+        <v>225</v>
+      </c>
+      <c r="K238" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="239" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A239" t="s">
+        <v>213</v>
+      </c>
+      <c r="B239" t="s">
+        <v>219</v>
+      </c>
+      <c r="C239" t="s">
+        <v>6</v>
+      </c>
+      <c r="D239" t="s">
+        <v>123</v>
+      </c>
+      <c r="E239">
+        <v>20260504</v>
+      </c>
+      <c r="F239">
+        <v>59.981255300000001</v>
+      </c>
+      <c r="G239">
+        <v>23.3646329</v>
+      </c>
+      <c r="H239" t="s">
+        <v>223</v>
+      </c>
+      <c r="I239" t="s">
+        <v>224</v>
+      </c>
+      <c r="J239" t="s">
+        <v>225</v>
+      </c>
+      <c r="K239" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="240" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A240" t="s">
+        <v>213</v>
+      </c>
+      <c r="B240" t="s">
+        <v>220</v>
+      </c>
+      <c r="C240" t="s">
+        <v>68</v>
+      </c>
+      <c r="D240" t="s">
+        <v>70</v>
+      </c>
+      <c r="E240">
+        <v>20260504</v>
+      </c>
+      <c r="H240" t="s">
+        <v>223</v>
+      </c>
+      <c r="I240" t="s">
+        <v>224</v>
+      </c>
+      <c r="J240" t="s">
+        <v>225</v>
+      </c>
+      <c r="K240" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="241" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A241" t="s">
+        <v>213</v>
+      </c>
+      <c r="B241" t="s">
+        <v>221</v>
+      </c>
+      <c r="C241" t="s">
+        <v>68</v>
+      </c>
+      <c r="D241" t="s">
+        <v>70</v>
+      </c>
+      <c r="E241">
+        <v>20260504</v>
+      </c>
+      <c r="H241" t="s">
+        <v>223</v>
+      </c>
+      <c r="I241" t="s">
+        <v>224</v>
+      </c>
+      <c r="J241" t="s">
+        <v>225</v>
+      </c>
+      <c r="K241" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="242" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A242" t="s">
+        <v>213</v>
+      </c>
+      <c r="B242" t="s">
+        <v>222</v>
+      </c>
+      <c r="C242" t="s">
+        <v>68</v>
+      </c>
+      <c r="D242" t="s">
+        <v>70</v>
+      </c>
+      <c r="E242">
+        <v>20260504</v>
+      </c>
+      <c r="H242" t="s">
+        <v>223</v>
+      </c>
+      <c r="I242" t="s">
+        <v>224</v>
+      </c>
+      <c r="J242" t="s">
+        <v>225</v>
+      </c>
+      <c r="K242" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="243" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A243" t="s">
+        <v>226</v>
+      </c>
+      <c r="B243" t="s">
+        <v>227</v>
+      </c>
+      <c r="C243" t="s">
+        <v>3</v>
+      </c>
+      <c r="D243" t="s">
+        <v>70</v>
+      </c>
+      <c r="E243">
+        <v>20260504</v>
+      </c>
+      <c r="F243">
+        <v>59.852577599999996</v>
+      </c>
+      <c r="G243">
+        <v>23.068529099999999</v>
+      </c>
+      <c r="H243" t="s">
+        <v>236</v>
+      </c>
+      <c r="I243" t="s">
+        <v>237</v>
+      </c>
+      <c r="J243" t="s">
+        <v>225</v>
+      </c>
+      <c r="K243" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="244" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A244" t="s">
+        <v>226</v>
+      </c>
+      <c r="B244" t="s">
+        <v>227</v>
+      </c>
+      <c r="C244" t="s">
+        <v>6</v>
+      </c>
+      <c r="D244" t="s">
+        <v>123</v>
+      </c>
+      <c r="E244">
+        <v>20260504</v>
+      </c>
+      <c r="F244">
+        <v>59.852577599999996</v>
+      </c>
+      <c r="G244">
+        <v>23.068529099999999</v>
+      </c>
+      <c r="H244" t="s">
+        <v>236</v>
+      </c>
+      <c r="I244" t="s">
+        <v>237</v>
+      </c>
+      <c r="J244" t="s">
+        <v>225</v>
+      </c>
+      <c r="K244" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="245" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A245" t="s">
+        <v>226</v>
+      </c>
+      <c r="B245" t="s">
+        <v>228</v>
+      </c>
+      <c r="C245" t="s">
+        <v>3</v>
+      </c>
+      <c r="D245" t="s">
+        <v>70</v>
+      </c>
+      <c r="E245">
+        <v>20260504</v>
+      </c>
+      <c r="H245" t="s">
+        <v>236</v>
+      </c>
+      <c r="I245" t="s">
+        <v>237</v>
+      </c>
+      <c r="J245" t="s">
+        <v>225</v>
+      </c>
+      <c r="K245" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="246" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A246" t="s">
+        <v>226</v>
+      </c>
+      <c r="B246" t="s">
+        <v>228</v>
+      </c>
+      <c r="C246" t="s">
+        <v>6</v>
+      </c>
+      <c r="D246" t="s">
+        <v>123</v>
+      </c>
+      <c r="E246">
+        <v>20260504</v>
+      </c>
+      <c r="H246" t="s">
+        <v>236</v>
+      </c>
+      <c r="I246" t="s">
+        <v>237</v>
+      </c>
+      <c r="J246" t="s">
+        <v>225</v>
+      </c>
+      <c r="K246" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="247" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A247" t="s">
+        <v>226</v>
+      </c>
+      <c r="B247" t="s">
+        <v>229</v>
+      </c>
+      <c r="C247" t="s">
+        <v>3</v>
+      </c>
+      <c r="D247" t="s">
+        <v>70</v>
+      </c>
+      <c r="E247">
+        <v>20260504</v>
+      </c>
+      <c r="H247" t="s">
+        <v>236</v>
+      </c>
+      <c r="I247" t="s">
+        <v>237</v>
+      </c>
+      <c r="J247" t="s">
+        <v>225</v>
+      </c>
+      <c r="K247" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="248" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A248" t="s">
+        <v>226</v>
+      </c>
+      <c r="B248" t="s">
+        <v>229</v>
+      </c>
+      <c r="C248" t="s">
+        <v>6</v>
+      </c>
+      <c r="D248" t="s">
+        <v>123</v>
+      </c>
+      <c r="E248">
+        <v>20260504</v>
+      </c>
+      <c r="H248" t="s">
+        <v>236</v>
+      </c>
+      <c r="I248" t="s">
+        <v>237</v>
+      </c>
+      <c r="J248" t="s">
+        <v>225</v>
+      </c>
+      <c r="K248" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="249" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A249" t="s">
+        <v>226</v>
+      </c>
+      <c r="B249" t="s">
+        <v>230</v>
+      </c>
+      <c r="C249" t="s">
+        <v>3</v>
+      </c>
+      <c r="D249" t="s">
+        <v>70</v>
+      </c>
+      <c r="E249">
+        <v>20260504</v>
+      </c>
+      <c r="H249" t="s">
+        <v>236</v>
+      </c>
+      <c r="I249" t="s">
+        <v>237</v>
+      </c>
+      <c r="J249" t="s">
+        <v>225</v>
+      </c>
+      <c r="K249" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="250" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A250" t="s">
+        <v>226</v>
+      </c>
+      <c r="B250" t="s">
+        <v>230</v>
+      </c>
+      <c r="C250" t="s">
+        <v>6</v>
+      </c>
+      <c r="D250" t="s">
+        <v>123</v>
+      </c>
+      <c r="E250">
+        <v>20260504</v>
+      </c>
+      <c r="H250" t="s">
+        <v>236</v>
+      </c>
+      <c r="I250" t="s">
+        <v>237</v>
+      </c>
+      <c r="J250" t="s">
+        <v>225</v>
+      </c>
+      <c r="K250" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="251" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A251" t="s">
+        <v>226</v>
+      </c>
+      <c r="B251" t="s">
+        <v>231</v>
+      </c>
+      <c r="C251" t="s">
+        <v>3</v>
+      </c>
+      <c r="D251" t="s">
+        <v>70</v>
+      </c>
+      <c r="E251">
+        <v>20260504</v>
+      </c>
+      <c r="H251" t="s">
+        <v>236</v>
+      </c>
+      <c r="I251" t="s">
+        <v>237</v>
+      </c>
+      <c r="J251" t="s">
+        <v>225</v>
+      </c>
+      <c r="K251" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="252" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A252" t="s">
+        <v>226</v>
+      </c>
+      <c r="B252" t="s">
+        <v>231</v>
+      </c>
+      <c r="C252" t="s">
+        <v>6</v>
+      </c>
+      <c r="D252" t="s">
+        <v>123</v>
+      </c>
+      <c r="E252">
+        <v>20260504</v>
+      </c>
+      <c r="H252" t="s">
+        <v>236</v>
+      </c>
+      <c r="I252" t="s">
+        <v>237</v>
+      </c>
+      <c r="J252" t="s">
+        <v>225</v>
+      </c>
+      <c r="K252" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="253" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A253" t="s">
+        <v>226</v>
+      </c>
+      <c r="B253" t="s">
+        <v>232</v>
+      </c>
+      <c r="C253" t="s">
+        <v>3</v>
+      </c>
+      <c r="D253" t="s">
+        <v>70</v>
+      </c>
+      <c r="E253">
+        <v>20260504</v>
+      </c>
+      <c r="F253">
+        <v>59.852385499999997</v>
+      </c>
+      <c r="G253">
+        <v>23.068426800000001</v>
+      </c>
+      <c r="H253" t="s">
+        <v>236</v>
+      </c>
+      <c r="I253" t="s">
+        <v>237</v>
+      </c>
+      <c r="J253" t="s">
+        <v>225</v>
+      </c>
+      <c r="K253" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="254" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A254" t="s">
+        <v>226</v>
+      </c>
+      <c r="B254" t="s">
+        <v>232</v>
+      </c>
+      <c r="C254" t="s">
+        <v>6</v>
+      </c>
+      <c r="D254" t="s">
+        <v>123</v>
+      </c>
+      <c r="E254">
+        <v>20260504</v>
+      </c>
+      <c r="F254">
+        <v>59.852385499999997</v>
+      </c>
+      <c r="G254">
+        <v>23.068426800000001</v>
+      </c>
+      <c r="H254" t="s">
+        <v>236</v>
+      </c>
+      <c r="I254" t="s">
+        <v>237</v>
+      </c>
+      <c r="J254" t="s">
+        <v>225</v>
+      </c>
+      <c r="K254" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="255" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A255" t="s">
+        <v>226</v>
+      </c>
+      <c r="B255" t="s">
+        <v>233</v>
+      </c>
+      <c r="C255" t="s">
+        <v>68</v>
+      </c>
+      <c r="D255" t="s">
+        <v>70</v>
+      </c>
+      <c r="E255">
+        <v>20260504</v>
+      </c>
+      <c r="H255" t="s">
+        <v>236</v>
+      </c>
+      <c r="I255" t="s">
+        <v>237</v>
+      </c>
+      <c r="J255" t="s">
+        <v>225</v>
+      </c>
+      <c r="K255" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="256" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A256" t="s">
+        <v>226</v>
+      </c>
+      <c r="B256" t="s">
+        <v>234</v>
+      </c>
+      <c r="C256" t="s">
+        <v>68</v>
+      </c>
+      <c r="D256" t="s">
+        <v>70</v>
+      </c>
+      <c r="E256">
+        <v>20260504</v>
+      </c>
+      <c r="H256" t="s">
+        <v>236</v>
+      </c>
+      <c r="I256" t="s">
+        <v>237</v>
+      </c>
+      <c r="J256" t="s">
+        <v>225</v>
+      </c>
+      <c r="K256" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="257" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A257" t="s">
+        <v>226</v>
+      </c>
+      <c r="B257" t="s">
+        <v>235</v>
+      </c>
+      <c r="C257" t="s">
+        <v>68</v>
+      </c>
+      <c r="D257" t="s">
+        <v>70</v>
+      </c>
+      <c r="E257">
+        <v>20260504</v>
+      </c>
+      <c r="H257" t="s">
+        <v>236</v>
+      </c>
+      <c r="I257" t="s">
+        <v>237</v>
+      </c>
+      <c r="J257" t="s">
+        <v>225</v>
+      </c>
+      <c r="K257" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="258" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A258" t="s">
+        <v>238</v>
+      </c>
+      <c r="B258" t="s">
+        <v>239</v>
+      </c>
+      <c r="C258" t="s">
+        <v>3</v>
+      </c>
+      <c r="D258" t="s">
+        <v>70</v>
+      </c>
+      <c r="E258">
+        <v>20260505</v>
+      </c>
+      <c r="F258">
+        <v>60.002580000000002</v>
+      </c>
+      <c r="G258">
+        <v>23.175820099999999</v>
+      </c>
+      <c r="H258" t="s">
+        <v>248</v>
+      </c>
+      <c r="I258" t="s">
+        <v>249</v>
+      </c>
+      <c r="J258" t="s">
+        <v>225</v>
+      </c>
+      <c r="K258" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="259" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A259" t="s">
+        <v>238</v>
+      </c>
+      <c r="B259" t="s">
+        <v>239</v>
+      </c>
+      <c r="C259" t="s">
+        <v>6</v>
+      </c>
+      <c r="D259" t="s">
+        <v>123</v>
+      </c>
+      <c r="E259">
+        <v>20260505</v>
+      </c>
+      <c r="F259">
+        <v>60.002580000000002</v>
+      </c>
+      <c r="G259">
+        <v>23.175820099999999</v>
+      </c>
+      <c r="H259" t="s">
+        <v>248</v>
+      </c>
+      <c r="I259" t="s">
+        <v>249</v>
+      </c>
+      <c r="J259" t="s">
+        <v>225</v>
+      </c>
+      <c r="K259" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="260" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A260" t="s">
+        <v>238</v>
+      </c>
+      <c r="B260" t="s">
+        <v>240</v>
+      </c>
+      <c r="C260" t="s">
+        <v>3</v>
+      </c>
+      <c r="D260" t="s">
+        <v>70</v>
+      </c>
+      <c r="E260">
+        <v>20260505</v>
+      </c>
+      <c r="H260" t="s">
+        <v>248</v>
+      </c>
+      <c r="I260" t="s">
+        <v>249</v>
+      </c>
+      <c r="J260" t="s">
+        <v>225</v>
+      </c>
+      <c r="K260" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="261" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A261" t="s">
+        <v>238</v>
+      </c>
+      <c r="B261" t="s">
+        <v>240</v>
+      </c>
+      <c r="C261" t="s">
+        <v>6</v>
+      </c>
+      <c r="D261" t="s">
+        <v>123</v>
+      </c>
+      <c r="E261">
+        <v>20260505</v>
+      </c>
+      <c r="H261" t="s">
+        <v>248</v>
+      </c>
+      <c r="I261" t="s">
+        <v>249</v>
+      </c>
+      <c r="J261" t="s">
+        <v>225</v>
+      </c>
+      <c r="K261" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="262" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A262" t="s">
+        <v>238</v>
+      </c>
+      <c r="B262" t="s">
+        <v>241</v>
+      </c>
+      <c r="C262" t="s">
+        <v>3</v>
+      </c>
+      <c r="D262" t="s">
+        <v>70</v>
+      </c>
+      <c r="E262">
+        <v>20260505</v>
+      </c>
+      <c r="H262" t="s">
+        <v>248</v>
+      </c>
+      <c r="I262" t="s">
+        <v>249</v>
+      </c>
+      <c r="J262" t="s">
+        <v>225</v>
+      </c>
+      <c r="K262" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="263" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A263" t="s">
+        <v>238</v>
+      </c>
+      <c r="B263" t="s">
+        <v>241</v>
+      </c>
+      <c r="C263" t="s">
+        <v>6</v>
+      </c>
+      <c r="D263" t="s">
+        <v>123</v>
+      </c>
+      <c r="E263">
+        <v>20260505</v>
+      </c>
+      <c r="H263" t="s">
+        <v>248</v>
+      </c>
+      <c r="I263" t="s">
+        <v>249</v>
+      </c>
+      <c r="J263" t="s">
+        <v>225</v>
+      </c>
+      <c r="K263" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="264" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A264" t="s">
+        <v>238</v>
+      </c>
+      <c r="B264" t="s">
+        <v>242</v>
+      </c>
+      <c r="C264" t="s">
+        <v>3</v>
+      </c>
+      <c r="D264" t="s">
+        <v>70</v>
+      </c>
+      <c r="E264">
+        <v>20260505</v>
+      </c>
+      <c r="H264" t="s">
+        <v>248</v>
+      </c>
+      <c r="I264" t="s">
+        <v>249</v>
+      </c>
+      <c r="J264" t="s">
+        <v>225</v>
+      </c>
+      <c r="K264" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="265" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A265" t="s">
+        <v>238</v>
+      </c>
+      <c r="B265" t="s">
+        <v>242</v>
+      </c>
+      <c r="C265" t="s">
+        <v>6</v>
+      </c>
+      <c r="D265" t="s">
+        <v>123</v>
+      </c>
+      <c r="E265">
+        <v>20260505</v>
+      </c>
+      <c r="H265" t="s">
+        <v>248</v>
+      </c>
+      <c r="I265" t="s">
+        <v>249</v>
+      </c>
+      <c r="J265" t="s">
+        <v>225</v>
+      </c>
+      <c r="K265" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="266" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A266" t="s">
+        <v>238</v>
+      </c>
+      <c r="B266" t="s">
+        <v>243</v>
+      </c>
+      <c r="C266" t="s">
+        <v>3</v>
+      </c>
+      <c r="D266" t="s">
+        <v>70</v>
+      </c>
+      <c r="E266">
+        <v>20260505</v>
+      </c>
+      <c r="H266" t="s">
+        <v>248</v>
+      </c>
+      <c r="I266" t="s">
+        <v>249</v>
+      </c>
+      <c r="J266" t="s">
+        <v>225</v>
+      </c>
+      <c r="K266" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="267" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A267" t="s">
+        <v>238</v>
+      </c>
+      <c r="B267" t="s">
+        <v>243</v>
+      </c>
+      <c r="C267" t="s">
+        <v>6</v>
+      </c>
+      <c r="D267" t="s">
+        <v>123</v>
+      </c>
+      <c r="E267">
+        <v>20260505</v>
+      </c>
+      <c r="H267" t="s">
+        <v>248</v>
+      </c>
+      <c r="I267" t="s">
+        <v>249</v>
+      </c>
+      <c r="J267" t="s">
+        <v>225</v>
+      </c>
+      <c r="K267" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="268" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A268" t="s">
+        <v>238</v>
+      </c>
+      <c r="B268" t="s">
+        <v>244</v>
+      </c>
+      <c r="C268" t="s">
+        <v>3</v>
+      </c>
+      <c r="D268" t="s">
+        <v>70</v>
+      </c>
+      <c r="E268">
+        <v>20260505</v>
+      </c>
+      <c r="F268">
+        <v>60.002500099999999</v>
+      </c>
+      <c r="G268">
+        <v>23.176219400000001</v>
+      </c>
+      <c r="H268" t="s">
+        <v>248</v>
+      </c>
+      <c r="I268" t="s">
+        <v>249</v>
+      </c>
+      <c r="J268" t="s">
+        <v>225</v>
+      </c>
+      <c r="K268" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="269" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A269" t="s">
+        <v>238</v>
+      </c>
+      <c r="B269" t="s">
+        <v>244</v>
+      </c>
+      <c r="C269" t="s">
+        <v>6</v>
+      </c>
+      <c r="D269" t="s">
+        <v>123</v>
+      </c>
+      <c r="E269">
+        <v>20260505</v>
+      </c>
+      <c r="F269">
+        <v>60.002500099999999</v>
+      </c>
+      <c r="G269">
+        <v>23.176219400000001</v>
+      </c>
+      <c r="H269" t="s">
+        <v>248</v>
+      </c>
+      <c r="I269" t="s">
+        <v>249</v>
+      </c>
+      <c r="J269" t="s">
+        <v>225</v>
+      </c>
+      <c r="K269" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="270" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A270" t="s">
+        <v>238</v>
+      </c>
+      <c r="B270" t="s">
+        <v>245</v>
+      </c>
+      <c r="C270" t="s">
+        <v>68</v>
+      </c>
+      <c r="D270" t="s">
+        <v>70</v>
+      </c>
+      <c r="E270">
+        <v>20260505</v>
+      </c>
+      <c r="H270" t="s">
+        <v>248</v>
+      </c>
+      <c r="I270" t="s">
+        <v>249</v>
+      </c>
+      <c r="J270" t="s">
+        <v>225</v>
+      </c>
+      <c r="K270" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="271" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A271" t="s">
+        <v>238</v>
+      </c>
+      <c r="B271" t="s">
+        <v>246</v>
+      </c>
+      <c r="C271" t="s">
+        <v>68</v>
+      </c>
+      <c r="D271" t="s">
+        <v>70</v>
+      </c>
+      <c r="E271">
+        <v>20260505</v>
+      </c>
+      <c r="H271" t="s">
+        <v>248</v>
+      </c>
+      <c r="I271" t="s">
+        <v>249</v>
+      </c>
+      <c r="J271" t="s">
+        <v>225</v>
+      </c>
+      <c r="K271" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="272" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A272" t="s">
+        <v>238</v>
+      </c>
+      <c r="B272" t="s">
+        <v>247</v>
+      </c>
+      <c r="C272" t="s">
+        <v>68</v>
+      </c>
+      <c r="D272" t="s">
+        <v>70</v>
+      </c>
+      <c r="E272">
+        <v>20260505</v>
+      </c>
+      <c r="H272" t="s">
+        <v>248</v>
+      </c>
+      <c r="I272" t="s">
+        <v>249</v>
+      </c>
+      <c r="J272" t="s">
+        <v>225</v>
+      </c>
+      <c r="K272" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="273" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A273" t="s">
+        <v>250</v>
+      </c>
+      <c r="B273" t="s">
+        <v>251</v>
+      </c>
+      <c r="C273" t="s">
+        <v>3</v>
+      </c>
+      <c r="D273" t="s">
+        <v>70</v>
+      </c>
+      <c r="E273">
+        <v>20260505</v>
+      </c>
+      <c r="F273">
+        <v>60.001221399999999</v>
+      </c>
+      <c r="G273">
+        <v>23.171687500000001</v>
+      </c>
+      <c r="H273" t="s">
+        <v>260</v>
+      </c>
+      <c r="I273" t="s">
+        <v>261</v>
+      </c>
+      <c r="J273" t="s">
+        <v>225</v>
+      </c>
+      <c r="K273" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="274" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A274" t="s">
+        <v>250</v>
+      </c>
+      <c r="B274" t="s">
+        <v>251</v>
+      </c>
+      <c r="C274" t="s">
+        <v>6</v>
+      </c>
+      <c r="D274" t="s">
+        <v>123</v>
+      </c>
+      <c r="E274">
+        <v>20260505</v>
+      </c>
+      <c r="F274">
+        <v>60.001221399999999</v>
+      </c>
+      <c r="G274">
+        <v>23.171687500000001</v>
+      </c>
+      <c r="H274" t="s">
+        <v>260</v>
+      </c>
+      <c r="I274" t="s">
+        <v>261</v>
+      </c>
+      <c r="J274" t="s">
+        <v>225</v>
+      </c>
+      <c r="K274" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="275" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A275" t="s">
+        <v>250</v>
+      </c>
+      <c r="B275" t="s">
+        <v>252</v>
+      </c>
+      <c r="C275" t="s">
+        <v>3</v>
+      </c>
+      <c r="D275" t="s">
+        <v>70</v>
+      </c>
+      <c r="E275">
+        <v>20260505</v>
+      </c>
+      <c r="H275" t="s">
+        <v>260</v>
+      </c>
+      <c r="I275" t="s">
+        <v>261</v>
+      </c>
+      <c r="J275" t="s">
+        <v>225</v>
+      </c>
+      <c r="K275" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="276" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A276" t="s">
+        <v>250</v>
+      </c>
+      <c r="B276" t="s">
+        <v>252</v>
+      </c>
+      <c r="C276" t="s">
+        <v>6</v>
+      </c>
+      <c r="D276" t="s">
+        <v>123</v>
+      </c>
+      <c r="E276">
+        <v>20260505</v>
+      </c>
+      <c r="H276" t="s">
+        <v>260</v>
+      </c>
+      <c r="I276" t="s">
+        <v>261</v>
+      </c>
+      <c r="J276" t="s">
+        <v>225</v>
+      </c>
+      <c r="K276" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="277" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A277" t="s">
+        <v>250</v>
+      </c>
+      <c r="B277" t="s">
+        <v>253</v>
+      </c>
+      <c r="C277" t="s">
+        <v>3</v>
+      </c>
+      <c r="D277" t="s">
+        <v>70</v>
+      </c>
+      <c r="E277">
+        <v>20260505</v>
+      </c>
+      <c r="H277" t="s">
+        <v>260</v>
+      </c>
+      <c r="I277" t="s">
+        <v>261</v>
+      </c>
+      <c r="J277" t="s">
+        <v>225</v>
+      </c>
+      <c r="K277" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="278" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A278" t="s">
+        <v>250</v>
+      </c>
+      <c r="B278" t="s">
+        <v>253</v>
+      </c>
+      <c r="C278" t="s">
+        <v>6</v>
+      </c>
+      <c r="D278" t="s">
+        <v>123</v>
+      </c>
+      <c r="E278">
+        <v>20260505</v>
+      </c>
+      <c r="H278" t="s">
+        <v>260</v>
+      </c>
+      <c r="I278" t="s">
+        <v>261</v>
+      </c>
+      <c r="J278" t="s">
+        <v>225</v>
+      </c>
+      <c r="K278" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="279" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A279" t="s">
+        <v>250</v>
+      </c>
+      <c r="B279" t="s">
+        <v>254</v>
+      </c>
+      <c r="C279" t="s">
+        <v>3</v>
+      </c>
+      <c r="D279" t="s">
+        <v>70</v>
+      </c>
+      <c r="E279">
+        <v>20260505</v>
+      </c>
+      <c r="H279" t="s">
+        <v>260</v>
+      </c>
+      <c r="I279" t="s">
+        <v>261</v>
+      </c>
+      <c r="J279" t="s">
+        <v>225</v>
+      </c>
+      <c r="K279" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="280" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A280" t="s">
+        <v>250</v>
+      </c>
+      <c r="B280" t="s">
+        <v>254</v>
+      </c>
+      <c r="C280" t="s">
+        <v>6</v>
+      </c>
+      <c r="D280" t="s">
+        <v>123</v>
+      </c>
+      <c r="E280">
+        <v>20260505</v>
+      </c>
+      <c r="H280" t="s">
+        <v>260</v>
+      </c>
+      <c r="I280" t="s">
+        <v>261</v>
+      </c>
+      <c r="J280" t="s">
+        <v>225</v>
+      </c>
+      <c r="K280" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="281" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A281" t="s">
+        <v>250</v>
+      </c>
+      <c r="B281" t="s">
+        <v>255</v>
+      </c>
+      <c r="C281" t="s">
+        <v>3</v>
+      </c>
+      <c r="D281" t="s">
+        <v>70</v>
+      </c>
+      <c r="E281">
+        <v>20260505</v>
+      </c>
+      <c r="H281" t="s">
+        <v>260</v>
+      </c>
+      <c r="I281" t="s">
+        <v>261</v>
+      </c>
+      <c r="J281" t="s">
+        <v>225</v>
+      </c>
+      <c r="K281" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="282" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A282" t="s">
+        <v>250</v>
+      </c>
+      <c r="B282" t="s">
+        <v>255</v>
+      </c>
+      <c r="C282" t="s">
+        <v>6</v>
+      </c>
+      <c r="D282" t="s">
+        <v>123</v>
+      </c>
+      <c r="E282">
+        <v>20260505</v>
+      </c>
+      <c r="H282" t="s">
+        <v>260</v>
+      </c>
+      <c r="I282" t="s">
+        <v>261</v>
+      </c>
+      <c r="J282" t="s">
+        <v>225</v>
+      </c>
+      <c r="K282" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="283" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A283" t="s">
+        <v>250</v>
+      </c>
+      <c r="B283" t="s">
+        <v>256</v>
+      </c>
+      <c r="C283" t="s">
+        <v>3</v>
+      </c>
+      <c r="D283" t="s">
+        <v>70</v>
+      </c>
+      <c r="E283">
+        <v>20260505</v>
+      </c>
+      <c r="F283">
+        <v>60.001263600000001</v>
+      </c>
+      <c r="G283">
+        <v>23.171288499999999</v>
+      </c>
+      <c r="H283" t="s">
+        <v>260</v>
+      </c>
+      <c r="I283" t="s">
+        <v>261</v>
+      </c>
+      <c r="J283" t="s">
+        <v>225</v>
+      </c>
+      <c r="K283" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="284" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A284" t="s">
+        <v>250</v>
+      </c>
+      <c r="B284" t="s">
+        <v>256</v>
+      </c>
+      <c r="C284" t="s">
+        <v>6</v>
+      </c>
+      <c r="D284" t="s">
+        <v>123</v>
+      </c>
+      <c r="E284">
+        <v>20260505</v>
+      </c>
+      <c r="F284">
+        <v>60.001263600000001</v>
+      </c>
+      <c r="G284">
+        <v>23.171288499999999</v>
+      </c>
+      <c r="H284" t="s">
+        <v>260</v>
+      </c>
+      <c r="I284" t="s">
+        <v>261</v>
+      </c>
+      <c r="J284" t="s">
+        <v>225</v>
+      </c>
+      <c r="K284" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="285" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A285" t="s">
+        <v>250</v>
+      </c>
+      <c r="B285" t="s">
+        <v>257</v>
+      </c>
+      <c r="C285" t="s">
+        <v>68</v>
+      </c>
+      <c r="D285" t="s">
+        <v>70</v>
+      </c>
+      <c r="E285">
+        <v>20260505</v>
+      </c>
+      <c r="H285" t="s">
+        <v>260</v>
+      </c>
+      <c r="I285" t="s">
+        <v>261</v>
+      </c>
+      <c r="J285" t="s">
+        <v>225</v>
+      </c>
+      <c r="K285" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="286" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A286" t="s">
+        <v>250</v>
+      </c>
+      <c r="B286" t="s">
+        <v>258</v>
+      </c>
+      <c r="C286" t="s">
+        <v>68</v>
+      </c>
+      <c r="D286" t="s">
+        <v>70</v>
+      </c>
+      <c r="E286">
+        <v>20260505</v>
+      </c>
+      <c r="H286" t="s">
+        <v>260</v>
+      </c>
+      <c r="I286" t="s">
+        <v>261</v>
+      </c>
+      <c r="J286" t="s">
+        <v>225</v>
+      </c>
+      <c r="K286" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="287" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A287" t="s">
+        <v>250</v>
+      </c>
+      <c r="B287" t="s">
+        <v>259</v>
+      </c>
+      <c r="C287" t="s">
+        <v>68</v>
+      </c>
+      <c r="D287" t="s">
+        <v>70</v>
+      </c>
+      <c r="E287">
+        <v>20260505</v>
+      </c>
+      <c r="H287" t="s">
+        <v>260</v>
+      </c>
+      <c r="I287" t="s">
+        <v>261</v>
+      </c>
+      <c r="J287" t="s">
+        <v>225</v>
+      </c>
+      <c r="K287" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="288" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A288" t="s">
+        <v>262</v>
+      </c>
+      <c r="B288" t="s">
+        <v>263</v>
+      </c>
+      <c r="C288" t="s">
+        <v>3</v>
+      </c>
+      <c r="D288" t="s">
+        <v>70</v>
+      </c>
+      <c r="E288">
+        <v>20260506</v>
+      </c>
+      <c r="F288">
+        <v>60.039135600000002</v>
+      </c>
+      <c r="G288">
+        <v>23.2851848</v>
+      </c>
+      <c r="H288" t="s">
+        <v>248</v>
+      </c>
+      <c r="J288" t="s">
+        <v>225</v>
+      </c>
+      <c r="K288" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="289" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A289" t="s">
+        <v>262</v>
+      </c>
+      <c r="B289" t="s">
+        <v>263</v>
+      </c>
+      <c r="C289" t="s">
+        <v>6</v>
+      </c>
+      <c r="D289" t="s">
+        <v>123</v>
+      </c>
+      <c r="E289">
+        <v>20260506</v>
+      </c>
+      <c r="F289">
+        <v>60.039135600000002</v>
+      </c>
+      <c r="G289">
+        <v>23.2851848</v>
+      </c>
+      <c r="H289" t="s">
+        <v>248</v>
+      </c>
+      <c r="J289" t="s">
+        <v>225</v>
+      </c>
+      <c r="K289" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="290" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A290" t="s">
+        <v>262</v>
+      </c>
+      <c r="B290" t="s">
+        <v>264</v>
+      </c>
+      <c r="C290" t="s">
+        <v>3</v>
+      </c>
+      <c r="D290" t="s">
+        <v>70</v>
+      </c>
+      <c r="E290">
+        <v>20260506</v>
+      </c>
+      <c r="H290" t="s">
+        <v>248</v>
+      </c>
+      <c r="J290" t="s">
+        <v>225</v>
+      </c>
+      <c r="K290" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="291" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A291" t="s">
+        <v>262</v>
+      </c>
+      <c r="B291" t="s">
+        <v>264</v>
+      </c>
+      <c r="C291" t="s">
+        <v>6</v>
+      </c>
+      <c r="D291" t="s">
+        <v>123</v>
+      </c>
+      <c r="E291">
+        <v>20260506</v>
+      </c>
+      <c r="H291" t="s">
+        <v>248</v>
+      </c>
+      <c r="J291" t="s">
+        <v>225</v>
+      </c>
+      <c r="K291" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="292" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A292" t="s">
+        <v>262</v>
+      </c>
+      <c r="B292" t="s">
+        <v>265</v>
+      </c>
+      <c r="C292" t="s">
+        <v>3</v>
+      </c>
+      <c r="D292" t="s">
+        <v>70</v>
+      </c>
+      <c r="E292">
+        <v>20260506</v>
+      </c>
+      <c r="H292" t="s">
+        <v>248</v>
+      </c>
+      <c r="J292" t="s">
+        <v>225</v>
+      </c>
+      <c r="K292" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="293" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A293" t="s">
+        <v>262</v>
+      </c>
+      <c r="B293" t="s">
+        <v>265</v>
+      </c>
+      <c r="C293" t="s">
+        <v>6</v>
+      </c>
+      <c r="D293" t="s">
+        <v>123</v>
+      </c>
+      <c r="E293">
+        <v>20260506</v>
+      </c>
+      <c r="H293" t="s">
+        <v>248</v>
+      </c>
+      <c r="J293" t="s">
+        <v>225</v>
+      </c>
+      <c r="K293" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="294" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A294" t="s">
+        <v>262</v>
+      </c>
+      <c r="B294" t="s">
+        <v>266</v>
+      </c>
+      <c r="C294" t="s">
+        <v>3</v>
+      </c>
+      <c r="D294" t="s">
+        <v>70</v>
+      </c>
+      <c r="E294">
+        <v>20260506</v>
+      </c>
+      <c r="H294" t="s">
+        <v>248</v>
+      </c>
+      <c r="J294" t="s">
+        <v>225</v>
+      </c>
+      <c r="K294" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="295" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A295" t="s">
+        <v>262</v>
+      </c>
+      <c r="B295" t="s">
+        <v>266</v>
+      </c>
+      <c r="C295" t="s">
+        <v>6</v>
+      </c>
+      <c r="D295" t="s">
+        <v>123</v>
+      </c>
+      <c r="E295">
+        <v>20260506</v>
+      </c>
+      <c r="H295" t="s">
+        <v>248</v>
+      </c>
+      <c r="J295" t="s">
+        <v>225</v>
+      </c>
+      <c r="K295" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="296" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A296" t="s">
+        <v>262</v>
+      </c>
+      <c r="B296" t="s">
+        <v>267</v>
+      </c>
+      <c r="C296" t="s">
+        <v>3</v>
+      </c>
+      <c r="D296" t="s">
+        <v>70</v>
+      </c>
+      <c r="E296">
+        <v>20260506</v>
+      </c>
+      <c r="H296" t="s">
+        <v>248</v>
+      </c>
+      <c r="J296" t="s">
+        <v>225</v>
+      </c>
+      <c r="K296" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="297" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A297" t="s">
+        <v>262</v>
+      </c>
+      <c r="B297" t="s">
+        <v>267</v>
+      </c>
+      <c r="C297" t="s">
+        <v>6</v>
+      </c>
+      <c r="D297" t="s">
+        <v>123</v>
+      </c>
+      <c r="E297">
+        <v>20260506</v>
+      </c>
+      <c r="H297" t="s">
+        <v>248</v>
+      </c>
+      <c r="J297" t="s">
+        <v>225</v>
+      </c>
+      <c r="K297" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="298" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A298" t="s">
+        <v>262</v>
+      </c>
+      <c r="B298" t="s">
+        <v>268</v>
+      </c>
+      <c r="C298" t="s">
+        <v>3</v>
+      </c>
+      <c r="D298" t="s">
+        <v>70</v>
+      </c>
+      <c r="E298">
+        <v>20260506</v>
+      </c>
+      <c r="F298">
+        <v>60.039266699999999</v>
+      </c>
+      <c r="G298">
+        <v>23.2847802</v>
+      </c>
+      <c r="H298" t="s">
+        <v>248</v>
+      </c>
+      <c r="J298" t="s">
+        <v>225</v>
+      </c>
+      <c r="K298" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="299" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A299" t="s">
+        <v>262</v>
+      </c>
+      <c r="B299" t="s">
+        <v>268</v>
+      </c>
+      <c r="C299" t="s">
+        <v>6</v>
+      </c>
+      <c r="D299" t="s">
+        <v>123</v>
+      </c>
+      <c r="E299">
+        <v>20260506</v>
+      </c>
+      <c r="F299">
+        <v>60.039266699999999</v>
+      </c>
+      <c r="G299">
+        <v>23.2847802</v>
+      </c>
+      <c r="H299" t="s">
+        <v>248</v>
+      </c>
+      <c r="J299" t="s">
+        <v>225</v>
+      </c>
+      <c r="K299" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="300" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A300" t="s">
+        <v>262</v>
+      </c>
+      <c r="B300" t="s">
+        <v>269</v>
+      </c>
+      <c r="C300" t="s">
+        <v>68</v>
+      </c>
+      <c r="D300" t="s">
+        <v>70</v>
+      </c>
+      <c r="E300">
+        <v>20260506</v>
+      </c>
+      <c r="H300" t="s">
+        <v>248</v>
+      </c>
+      <c r="J300" t="s">
+        <v>225</v>
+      </c>
+      <c r="K300" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="301" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A301" t="s">
+        <v>262</v>
+      </c>
+      <c r="B301" t="s">
+        <v>270</v>
+      </c>
+      <c r="C301" t="s">
+        <v>68</v>
+      </c>
+      <c r="D301" t="s">
+        <v>70</v>
+      </c>
+      <c r="E301">
+        <v>20260506</v>
+      </c>
+      <c r="H301" t="s">
+        <v>248</v>
+      </c>
+      <c r="J301" t="s">
+        <v>225</v>
+      </c>
+      <c r="K301" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="302" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A302" t="s">
+        <v>262</v>
+      </c>
+      <c r="B302" t="s">
+        <v>271</v>
+      </c>
+      <c r="C302" t="s">
+        <v>68</v>
+      </c>
+      <c r="D302" t="s">
+        <v>70</v>
+      </c>
+      <c r="E302">
+        <v>20260506</v>
+      </c>
+      <c r="H302" t="s">
+        <v>248</v>
+      </c>
+      <c r="J302" t="s">
+        <v>225</v>
+      </c>
+      <c r="K302" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="303" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A303" t="s">
+        <v>272</v>
+      </c>
+      <c r="B303" t="s">
+        <v>273</v>
+      </c>
+      <c r="C303" t="s">
+        <v>3</v>
+      </c>
+      <c r="D303" t="s">
+        <v>70</v>
+      </c>
+      <c r="E303">
+        <v>20260506</v>
+      </c>
+      <c r="F303">
+        <v>60.041592000000001</v>
+      </c>
+      <c r="G303">
+        <v>23.2581156</v>
+      </c>
+      <c r="H303" t="s">
+        <v>282</v>
+      </c>
+      <c r="J303" t="s">
+        <v>225</v>
+      </c>
+      <c r="K303" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="304" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A304" t="s">
+        <v>272</v>
+      </c>
+      <c r="B304" t="s">
+        <v>273</v>
+      </c>
+      <c r="C304" t="s">
+        <v>6</v>
+      </c>
+      <c r="D304" t="s">
+        <v>123</v>
+      </c>
+      <c r="E304">
+        <v>20260506</v>
+      </c>
+      <c r="F304">
+        <v>60.041592000000001</v>
+      </c>
+      <c r="G304">
+        <v>23.2581156</v>
+      </c>
+      <c r="H304" t="s">
+        <v>282</v>
+      </c>
+      <c r="J304" t="s">
+        <v>225</v>
+      </c>
+      <c r="K304" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="305" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A305" t="s">
+        <v>272</v>
+      </c>
+      <c r="B305" t="s">
+        <v>274</v>
+      </c>
+      <c r="C305" t="s">
+        <v>3</v>
+      </c>
+      <c r="D305" t="s">
+        <v>70</v>
+      </c>
+      <c r="E305">
+        <v>20260506</v>
+      </c>
+      <c r="H305" t="s">
+        <v>282</v>
+      </c>
+      <c r="J305" t="s">
+        <v>225</v>
+      </c>
+      <c r="K305" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="306" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A306" t="s">
+        <v>272</v>
+      </c>
+      <c r="B306" t="s">
+        <v>274</v>
+      </c>
+      <c r="C306" t="s">
+        <v>6</v>
+      </c>
+      <c r="D306" t="s">
+        <v>123</v>
+      </c>
+      <c r="E306">
+        <v>20260506</v>
+      </c>
+      <c r="H306" t="s">
+        <v>282</v>
+      </c>
+      <c r="J306" t="s">
+        <v>225</v>
+      </c>
+      <c r="K306" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="307" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A307" t="s">
+        <v>272</v>
+      </c>
+      <c r="B307" t="s">
+        <v>275</v>
+      </c>
+      <c r="C307" t="s">
+        <v>3</v>
+      </c>
+      <c r="D307" t="s">
+        <v>70</v>
+      </c>
+      <c r="E307">
+        <v>20260506</v>
+      </c>
+      <c r="H307" t="s">
+        <v>282</v>
+      </c>
+      <c r="J307" t="s">
+        <v>225</v>
+      </c>
+      <c r="K307" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="308" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A308" t="s">
+        <v>272</v>
+      </c>
+      <c r="B308" t="s">
+        <v>275</v>
+      </c>
+      <c r="C308" t="s">
+        <v>6</v>
+      </c>
+      <c r="D308" t="s">
+        <v>123</v>
+      </c>
+      <c r="E308">
+        <v>20260506</v>
+      </c>
+      <c r="H308" t="s">
+        <v>282</v>
+      </c>
+      <c r="J308" t="s">
+        <v>225</v>
+      </c>
+      <c r="K308" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="309" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A309" t="s">
+        <v>272</v>
+      </c>
+      <c r="B309" t="s">
+        <v>276</v>
+      </c>
+      <c r="C309" t="s">
+        <v>3</v>
+      </c>
+      <c r="D309" t="s">
+        <v>70</v>
+      </c>
+      <c r="E309">
+        <v>20260506</v>
+      </c>
+      <c r="H309" t="s">
+        <v>282</v>
+      </c>
+      <c r="J309" t="s">
+        <v>225</v>
+      </c>
+      <c r="K309" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="310" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A310" t="s">
+        <v>272</v>
+      </c>
+      <c r="B310" t="s">
+        <v>276</v>
+      </c>
+      <c r="C310" t="s">
+        <v>6</v>
+      </c>
+      <c r="D310" t="s">
+        <v>123</v>
+      </c>
+      <c r="E310">
+        <v>20260506</v>
+      </c>
+      <c r="H310" t="s">
+        <v>282</v>
+      </c>
+      <c r="J310" t="s">
+        <v>225</v>
+      </c>
+      <c r="K310" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="311" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A311" t="s">
+        <v>272</v>
+      </c>
+      <c r="B311" t="s">
+        <v>277</v>
+      </c>
+      <c r="C311" t="s">
+        <v>3</v>
+      </c>
+      <c r="D311" t="s">
+        <v>70</v>
+      </c>
+      <c r="E311">
+        <v>20260506</v>
+      </c>
+      <c r="H311" t="s">
+        <v>282</v>
+      </c>
+      <c r="J311" t="s">
+        <v>225</v>
+      </c>
+      <c r="K311" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="312" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A312" t="s">
+        <v>272</v>
+      </c>
+      <c r="B312" t="s">
+        <v>277</v>
+      </c>
+      <c r="C312" t="s">
+        <v>6</v>
+      </c>
+      <c r="D312" t="s">
+        <v>123</v>
+      </c>
+      <c r="E312">
+        <v>20260506</v>
+      </c>
+      <c r="H312" t="s">
+        <v>282</v>
+      </c>
+      <c r="J312" t="s">
+        <v>225</v>
+      </c>
+      <c r="K312" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="313" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A313" t="s">
+        <v>272</v>
+      </c>
+      <c r="B313" t="s">
+        <v>278</v>
+      </c>
+      <c r="C313" t="s">
+        <v>3</v>
+      </c>
+      <c r="D313" t="s">
+        <v>70</v>
+      </c>
+      <c r="E313">
+        <v>20260506</v>
+      </c>
+      <c r="F313">
+        <v>60.041712699999998</v>
+      </c>
+      <c r="G313">
+        <v>23.257658299999999</v>
+      </c>
+      <c r="H313" t="s">
+        <v>282</v>
+      </c>
+      <c r="J313" t="s">
+        <v>225</v>
+      </c>
+      <c r="K313" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="314" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A314" t="s">
+        <v>272</v>
+      </c>
+      <c r="B314" t="s">
+        <v>278</v>
+      </c>
+      <c r="C314" t="s">
+        <v>6</v>
+      </c>
+      <c r="D314" t="s">
+        <v>123</v>
+      </c>
+      <c r="E314">
+        <v>20260506</v>
+      </c>
+      <c r="F314">
+        <v>60.041712699999998</v>
+      </c>
+      <c r="G314">
+        <v>23.257658299999999</v>
+      </c>
+      <c r="H314" t="s">
+        <v>282</v>
+      </c>
+      <c r="J314" t="s">
+        <v>225</v>
+      </c>
+      <c r="K314" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="315" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A315" t="s">
+        <v>272</v>
+      </c>
+      <c r="B315" t="s">
+        <v>279</v>
+      </c>
+      <c r="C315" t="s">
+        <v>68</v>
+      </c>
+      <c r="D315" t="s">
+        <v>70</v>
+      </c>
+      <c r="E315">
+        <v>20260506</v>
+      </c>
+      <c r="H315" t="s">
+        <v>282</v>
+      </c>
+      <c r="J315" t="s">
+        <v>225</v>
+      </c>
+      <c r="K315" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="316" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A316" t="s">
+        <v>272</v>
+      </c>
+      <c r="B316" t="s">
+        <v>280</v>
+      </c>
+      <c r="C316" t="s">
+        <v>68</v>
+      </c>
+      <c r="D316" t="s">
+        <v>70</v>
+      </c>
+      <c r="E316">
+        <v>20260506</v>
+      </c>
+      <c r="H316" t="s">
+        <v>282</v>
+      </c>
+      <c r="J316" t="s">
+        <v>225</v>
+      </c>
+      <c r="K316" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="317" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A317" t="s">
+        <v>272</v>
+      </c>
+      <c r="B317" t="s">
+        <v>281</v>
+      </c>
+      <c r="C317" t="s">
+        <v>68</v>
+      </c>
+      <c r="D317" t="s">
+        <v>70</v>
+      </c>
+      <c r="E317">
+        <v>20260506</v>
+      </c>
+      <c r="H317" t="s">
+        <v>282</v>
+      </c>
+      <c r="J317" t="s">
+        <v>225</v>
+      </c>
+      <c r="K317" t="s">
+        <v>125</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I227" xr:uid="{1DCF7B1D-30EB-41FA-B0BA-2D9928994D79}"/>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>